<commit_message>
add destination infos tools based on internal Excel DB (tested verified OK)
</commit_message>
<xml_diff>
--- a/data/destinations_infos.xlsx
+++ b/data/destinations_infos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Vie Professionnelle\GitHub Projects\GENAI-travel-agent-openai-huggingfacespaces\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA24904-168A-41DB-9222-43C50E12330C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E195D4E-E295-4BFF-A4C2-AAD22C173725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -595,7 +595,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -623,7 +623,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -637,7 +637,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -651,7 +651,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -665,7 +665,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
@@ -679,7 +679,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -693,7 +693,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -735,7 +735,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
@@ -749,7 +749,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -763,7 +763,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>49</v>
       </c>
@@ -777,7 +777,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>52</v>
       </c>
@@ -791,7 +791,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>56</v>
       </c>
@@ -805,7 +805,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>59</v>
       </c>
@@ -819,7 +819,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>63</v>
       </c>
@@ -833,7 +833,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>67</v>
       </c>
@@ -847,7 +847,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>69</v>
       </c>

</xml_diff>